<commit_message>
Harden eval infra, fix task evaluators, and add rerun C1-C5 tooling
- Harden harness boundary, Slurm launch scripts, and local MCP servers
  (canvas pg router, calendar, google-sheets, notion pg client, youtube
  transcript, word file utils).
- Fix task evaluators and preprocess data (canvas-at-risk-intervention,
  ecommerce-commodity-impact, fetch-wc-yf-financial-excel-word-email).
- Add enroot image build/verify/postfix scripts and gcal eval linting.
- Add rerun C1-C5 Slurm launcher scripts and task order lists.
- Add single-vs-subagent comparison and artifact no-claim eval scripts.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tasks/finalpool/fetch-wc-yf-financial-excel-word-email/groundtruth_workspace/Yf_Financial_Report.xlsx
+++ b/tasks/finalpool/fetch-wc-yf-financial-excel-word-email/groundtruth_workspace/Yf_Financial_Report.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,22 +531,6 @@
         <v>289.65</v>
       </c>
       <c r="D6" t="n">
-        <v>5.3</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Watches</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>60.69</v>
-      </c>
-      <c r="C7" t="n">
-        <v>57.66</v>
-      </c>
-      <c r="D7" t="n">
         <v>5.3</v>
       </c>
     </row>
@@ -583,7 +567,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">

</xml_diff>